<commit_message>
Polish report headers and filenames
</commit_message>
<xml_diff>
--- a/report-saved-containers-summary.xlsx
+++ b/report-saved-containers-summary.xlsx
@@ -11,15 +11,21 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Container Report</t>
   </si>
   <si>
+    <t>Company</t>
+  </si>
+  <si>
+    <t>Skyinventories</t>
+  </si>
+  <si>
     <t>Generated At</t>
   </si>
   <si>
-    <t>02 Apr 2026, 09:11</t>
+    <t>02 Apr 2026, 09:24</t>
   </si>
   <si>
     <t>Mode</t>
@@ -53,13 +59,19 @@
   </si>
   <si>
     <t>Loading</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -80,8 +92,12 @@
       <b/>
       <color rgb="FFFFFFFF"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FF0F172A"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -101,6 +117,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1D4ED8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2E8F0"/>
       </patternFill>
     </fill>
   </fills>
@@ -131,7 +152,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -149,6 +170,10 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -490,7 +515,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
@@ -537,26 +562,45 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="6" t="s">
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+      <c r="B8" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="C8" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="4">
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="8">
         <v>1</v>
       </c>
     </row>

</xml_diff>